<commit_message>
Evénement Messager pour la Paix
</commit_message>
<xml_diff>
--- a/docs/Effet-de-Courroux-de-la-Terre.xlsx
+++ b/docs/Effet-de-Courroux-de-la-Terre.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leand\Documents\GitHub\Terre-de-Barons\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDE09308-F829-4EE0-A010-CF21EC02CDF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3426D6F-25AC-46D1-B13B-2D8E55DBD1B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-9120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Courroux de la Terre" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="10">
   <si>
     <t>proba</t>
   </si>
@@ -55,6 +55,18 @@
   <si>
     <t>à 2 joueurs</t>
   </si>
+  <si>
+    <t>3 positions tirées pour chaque événement calamité</t>
+  </si>
+  <si>
+    <t>2 positions tirées pour chaque événement calamité</t>
+  </si>
+  <si>
+    <t>prob cmp</t>
+  </si>
+  <si>
+    <t>1 position tirée pour chaque événement calamité</t>
+  </si>
 </sst>
 </file>
 
@@ -63,7 +75,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -72,6 +84,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -115,13 +135,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -403,330 +424,784 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:AC19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="12.140625" customWidth="1"/>
     <col min="3" max="3" width="17.140625" customWidth="1"/>
+    <col min="4" max="4" width="3.42578125" customWidth="1"/>
+    <col min="7" max="7" width="3.28515625" customWidth="1"/>
+    <col min="14" max="14" width="2.85546875" customWidth="1"/>
+    <col min="17" max="17" width="3.140625" customWidth="1"/>
+    <col min="24" max="24" width="3.28515625" customWidth="1"/>
+    <col min="27" max="27" width="2.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K1" t="s">
+        <v>7</v>
+      </c>
+      <c r="U1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E2" t="s">
         <v>4</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="3">
+      <c r="K2" t="s">
+        <v>3</v>
+      </c>
+      <c r="O2" t="s">
+        <v>4</v>
+      </c>
+      <c r="R2" t="s">
+        <v>5</v>
+      </c>
+      <c r="U2" t="s">
+        <v>3</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>4</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
         <v>1</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B4" s="3">
         <v>23</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C4" s="3">
         <v>33</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E4" s="3">
         <v>23</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F4" s="3">
         <v>33</v>
       </c>
-      <c r="H3" s="3">
+      <c r="H4" s="3">
         <v>23</v>
       </c>
-      <c r="I3" s="3">
+      <c r="I4" s="3">
         <v>33</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
+      <c r="K4" s="3">
+        <v>1</v>
+      </c>
+      <c r="L4" s="3">
+        <v>23</v>
+      </c>
+      <c r="M4" s="3">
+        <v>33</v>
+      </c>
+      <c r="O4" s="3">
+        <v>23</v>
+      </c>
+      <c r="P4" s="3">
+        <v>33</v>
+      </c>
+      <c r="R4" s="3">
+        <v>23</v>
+      </c>
+      <c r="S4" s="3">
+        <v>33</v>
+      </c>
+      <c r="U4" s="3">
+        <v>1</v>
+      </c>
+      <c r="V4" s="3">
+        <v>23</v>
+      </c>
+      <c r="W4" s="3">
+        <v>33</v>
+      </c>
+      <c r="Y4" s="3">
+        <v>23</v>
+      </c>
+      <c r="Z4" s="3">
+        <v>33</v>
+      </c>
+      <c r="AB4" s="3">
+        <v>23</v>
+      </c>
+      <c r="AC4" s="3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
         <v>2</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B5" s="3">
         <v>22</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C5" s="3">
         <v>32</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E5" s="3">
         <v>22</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F5" s="3">
         <v>32</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H5" s="3">
         <v>22</v>
       </c>
-      <c r="I4" s="3">
+      <c r="I5" s="3">
         <v>32</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="3">
+      <c r="K5" s="3">
+        <v>2</v>
+      </c>
+      <c r="L5" s="3">
+        <v>22</v>
+      </c>
+      <c r="M5" s="3">
+        <v>32</v>
+      </c>
+      <c r="O5" s="3">
+        <v>22</v>
+      </c>
+      <c r="P5" s="3">
+        <v>32</v>
+      </c>
+      <c r="R5" s="3">
+        <v>22</v>
+      </c>
+      <c r="S5" s="3">
+        <v>32</v>
+      </c>
+      <c r="U5" s="3">
+        <v>2</v>
+      </c>
+      <c r="V5" s="3">
+        <v>22</v>
+      </c>
+      <c r="W5" s="3">
+        <v>32</v>
+      </c>
+      <c r="Y5" s="3">
+        <v>22</v>
+      </c>
+      <c r="Z5" s="3">
+        <v>32</v>
+      </c>
+      <c r="AB5" s="3">
+        <v>22</v>
+      </c>
+      <c r="AC5" s="3">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A6" s="3">
         <v>3</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B6" s="3">
         <v>21</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C6" s="3">
         <v>31</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E6" s="3">
         <v>21</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F6" s="3">
         <v>31</v>
       </c>
-      <c r="H5" s="3">
+      <c r="H6" s="3">
         <v>21</v>
       </c>
-      <c r="I5" s="3">
+      <c r="I6" s="3">
         <v>31</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="3">
+      <c r="K6" s="3">
+        <v>3</v>
+      </c>
+      <c r="L6" s="3">
+        <v>21</v>
+      </c>
+      <c r="M6" s="3">
+        <v>31</v>
+      </c>
+      <c r="O6" s="3">
+        <v>21</v>
+      </c>
+      <c r="P6" s="3">
+        <v>31</v>
+      </c>
+      <c r="R6" s="3">
+        <v>21</v>
+      </c>
+      <c r="S6" s="3">
+        <v>31</v>
+      </c>
+      <c r="U6" s="3">
+        <v>3</v>
+      </c>
+      <c r="V6" s="3">
+        <v>21</v>
+      </c>
+      <c r="W6" s="3">
+        <v>31</v>
+      </c>
+      <c r="Y6" s="3">
+        <v>21</v>
+      </c>
+      <c r="Z6" s="3">
+        <v>31</v>
+      </c>
+      <c r="AB6" s="3"/>
+      <c r="AC6" s="3"/>
+    </row>
+    <row r="7" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A7" s="3">
         <v>4</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B7" s="3">
         <v>20</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C7" s="3">
         <v>30</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E7" s="3">
         <v>20</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F7" s="3">
         <v>30</v>
       </c>
-      <c r="H6" s="3">
+      <c r="H7" s="3">
         <v>20</v>
       </c>
-      <c r="I6" s="3">
+      <c r="I7" s="3">
         <v>30</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="3">
+      <c r="K7" s="3">
+        <v>4</v>
+      </c>
+      <c r="L7" s="3">
+        <v>20</v>
+      </c>
+      <c r="M7" s="3">
+        <v>30</v>
+      </c>
+      <c r="O7" s="3">
+        <v>20</v>
+      </c>
+      <c r="P7" s="3">
+        <v>30</v>
+      </c>
+      <c r="R7" s="3">
+        <v>20</v>
+      </c>
+      <c r="S7" s="3">
+        <v>30</v>
+      </c>
+      <c r="U7" s="3">
+        <v>4</v>
+      </c>
+      <c r="V7" s="3">
+        <v>20</v>
+      </c>
+      <c r="W7" s="3">
+        <v>30</v>
+      </c>
+      <c r="Y7" s="3"/>
+      <c r="Z7" s="3"/>
+      <c r="AB7" s="3"/>
+      <c r="AC7" s="3"/>
+    </row>
+    <row r="8" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A8" s="3">
         <v>5</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B8" s="3">
         <v>19</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C8" s="3">
         <v>29</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E8" s="3">
         <v>19</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F8" s="3">
         <v>29</v>
       </c>
-      <c r="H7" s="3">
+      <c r="H8" s="3">
         <v>19</v>
       </c>
-      <c r="I7" s="3">
+      <c r="I8" s="3">
         <v>29</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="3">
+      <c r="K8" s="3">
+        <v>5</v>
+      </c>
+      <c r="L8" s="3">
+        <v>19</v>
+      </c>
+      <c r="M8" s="3">
+        <v>29</v>
+      </c>
+      <c r="O8" s="3">
+        <v>19</v>
+      </c>
+      <c r="P8" s="3">
+        <v>29</v>
+      </c>
+      <c r="R8" s="3"/>
+      <c r="S8" s="3"/>
+      <c r="U8" s="3"/>
+      <c r="V8" s="3"/>
+      <c r="W8" s="3"/>
+      <c r="Y8" s="3"/>
+      <c r="Z8" s="3"/>
+      <c r="AB8" s="3"/>
+      <c r="AC8" s="3"/>
+    </row>
+    <row r="9" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A9" s="3">
         <v>6</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B9" s="3">
         <v>18</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C9" s="3">
         <v>28</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E9" s="3">
         <v>18</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F9" s="3">
         <v>28</v>
       </c>
-      <c r="H8" s="3">
+      <c r="H9" s="3">
         <v>18</v>
       </c>
-      <c r="I8" s="3">
+      <c r="I9" s="3">
         <v>28</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="3">
+      <c r="K9" s="3">
+        <v>6</v>
+      </c>
+      <c r="L9" s="3">
+        <v>18</v>
+      </c>
+      <c r="M9" s="3">
+        <v>28</v>
+      </c>
+      <c r="O9" s="3">
+        <v>18</v>
+      </c>
+      <c r="P9" s="3">
+        <v>28</v>
+      </c>
+      <c r="R9" s="3"/>
+      <c r="S9" s="3"/>
+      <c r="U9" s="3"/>
+      <c r="V9" s="3"/>
+      <c r="W9" s="3"/>
+      <c r="Y9" s="3"/>
+      <c r="Z9" s="3"/>
+      <c r="AB9" s="3"/>
+      <c r="AC9" s="3"/>
+    </row>
+    <row r="10" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A10" s="3">
         <v>7</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B10" s="3">
         <v>17</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C10" s="3">
         <v>27</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E10" s="3">
         <v>17</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F10" s="3">
         <v>27</v>
-      </c>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="3">
-        <v>8</v>
-      </c>
-      <c r="B10" s="3">
-        <v>16</v>
-      </c>
-      <c r="C10" s="3">
-        <v>26</v>
-      </c>
-      <c r="E10" s="3">
-        <v>16</v>
-      </c>
-      <c r="F10" s="3">
-        <v>26</v>
       </c>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K10" s="3">
+        <v>7</v>
+      </c>
+      <c r="L10" s="3">
+        <v>17</v>
+      </c>
+      <c r="M10" s="3">
+        <v>27</v>
+      </c>
+      <c r="O10" s="3"/>
+      <c r="P10" s="3"/>
+      <c r="R10" s="3"/>
+      <c r="S10" s="3"/>
+      <c r="U10" s="3"/>
+      <c r="V10" s="3"/>
+      <c r="W10" s="3"/>
+      <c r="Y10" s="3"/>
+      <c r="Z10" s="3"/>
+      <c r="AB10" s="3"/>
+      <c r="AC10" s="3"/>
+    </row>
+    <row r="11" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="3">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C11" s="3">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E11" s="3">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F11" s="3">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K11" s="3">
+        <v>8</v>
+      </c>
+      <c r="L11" s="3">
+        <v>16</v>
+      </c>
+      <c r="M11" s="3">
+        <v>26</v>
+      </c>
+      <c r="O11" s="3"/>
+      <c r="P11" s="3"/>
+      <c r="R11" s="3"/>
+      <c r="S11" s="3"/>
+      <c r="U11" s="3"/>
+      <c r="V11" s="3"/>
+      <c r="W11" s="3"/>
+      <c r="Y11" s="3"/>
+      <c r="Z11" s="3"/>
+      <c r="AB11" s="3"/>
+      <c r="AC11" s="3"/>
+    </row>
+    <row r="12" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" s="3">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C12" s="3">
-        <v>24</v>
-      </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="1"/>
+        <v>25</v>
+      </c>
+      <c r="E12" s="3">
+        <v>15</v>
+      </c>
+      <c r="F12" s="3">
+        <v>25</v>
+      </c>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K12" s="3"/>
+      <c r="L12" s="3"/>
+      <c r="M12" s="3"/>
+      <c r="O12" s="3"/>
+      <c r="P12" s="3"/>
+      <c r="R12" s="3"/>
+      <c r="S12" s="3"/>
+      <c r="U12" s="3"/>
+      <c r="V12" s="3"/>
+      <c r="W12" s="3"/>
+      <c r="Y12" s="3"/>
+      <c r="Z12" s="3"/>
+      <c r="AB12" s="3"/>
+      <c r="AC12" s="3"/>
+    </row>
+    <row r="13" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" s="3">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C13" s="3">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
-      <c r="G13" s="2"/>
+      <c r="G13" s="1"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K13" s="3"/>
+      <c r="L13" s="3"/>
+      <c r="M13" s="3"/>
+      <c r="O13" s="3"/>
+      <c r="P13" s="3"/>
+      <c r="Q13" s="1"/>
+      <c r="R13" s="3"/>
+      <c r="S13" s="3"/>
+      <c r="U13" s="3"/>
+      <c r="V13" s="3"/>
+      <c r="W13" s="3"/>
+      <c r="Y13" s="3"/>
+      <c r="Z13" s="3"/>
+      <c r="AA13" s="1"/>
+      <c r="AB13" s="3"/>
+      <c r="AC13" s="3"/>
+    </row>
+    <row r="14" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B14" s="3">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C14" s="3">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
+      <c r="G14" s="2"/>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="K14" s="3"/>
+      <c r="L14" s="3"/>
+      <c r="M14" s="3"/>
+      <c r="O14" s="3"/>
+      <c r="P14" s="3"/>
+      <c r="Q14" s="2"/>
+      <c r="R14" s="3"/>
+      <c r="S14" s="3"/>
+      <c r="U14" s="3"/>
+      <c r="V14" s="3"/>
+      <c r="W14" s="3"/>
+      <c r="Y14" s="3"/>
+      <c r="Z14" s="3"/>
+      <c r="AA14" s="2"/>
+      <c r="AB14" s="3"/>
+      <c r="AC14" s="3"/>
+    </row>
+    <row r="15" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A15" s="3">
+        <v>12</v>
+      </c>
+      <c r="B15" s="3">
+        <v>12</v>
+      </c>
+      <c r="C15" s="3">
+        <v>22</v>
+      </c>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="K15" s="3"/>
+      <c r="L15" s="3"/>
+      <c r="M15" s="3"/>
+      <c r="O15" s="3"/>
+      <c r="P15" s="3"/>
+      <c r="R15" s="3"/>
+      <c r="S15" s="3"/>
+      <c r="U15" s="3"/>
+      <c r="V15" s="3"/>
+      <c r="W15" s="3"/>
+      <c r="Y15" s="3"/>
+      <c r="Z15" s="3"/>
+      <c r="AB15" s="3"/>
+      <c r="AC15" s="3"/>
+    </row>
+    <row r="17" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>1</v>
       </c>
-      <c r="B16">
-        <f>PRODUCT(B3:B14)</f>
+      <c r="B17">
+        <f>PRODUCT(B4:B15)</f>
         <v>647647525324800</v>
       </c>
-      <c r="C16">
-        <f>PRODUCT(C3:C14)</f>
+      <c r="C17">
+        <f>PRODUCT(C4:C15)</f>
         <v>1.69958063987712E+17</v>
       </c>
-      <c r="E16">
-        <f>PRODUCT(E3:E14)</f>
+      <c r="E17">
+        <f>PRODUCT(E4:E15)</f>
         <v>296541907200</v>
       </c>
-      <c r="F16">
-        <f>PRODUCT(F3:F14)</f>
+      <c r="F17">
+        <f>PRODUCT(F4:F15)</f>
         <v>13995229248000</v>
       </c>
-      <c r="H16">
-        <f>PRODUCT(H3:H14)</f>
+      <c r="H17">
+        <f>PRODUCT(H4:H15)</f>
         <v>72681840</v>
       </c>
-      <c r="I16">
-        <f>PRODUCT(I3:I14)</f>
+      <c r="I17">
+        <f>PRODUCT(I4:I15)</f>
         <v>797448960</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="K17" t="s">
+        <v>1</v>
+      </c>
+      <c r="L17">
+        <f>PRODUCT(L4:L15)</f>
+        <v>19769460480</v>
+      </c>
+      <c r="M17">
+        <f>PRODUCT(M4:M15)</f>
+        <v>559809169920</v>
+      </c>
+      <c r="O17">
+        <f>PRODUCT(O4:O15)</f>
+        <v>72681840</v>
+      </c>
+      <c r="P17">
+        <f>PRODUCT(P4:P15)</f>
+        <v>797448960</v>
+      </c>
+      <c r="R17">
+        <f>PRODUCT(R4:R15)</f>
+        <v>212520</v>
+      </c>
+      <c r="S17">
+        <f>PRODUCT(S4:S15)</f>
+        <v>982080</v>
+      </c>
+      <c r="U17" t="s">
+        <v>1</v>
+      </c>
+      <c r="V17">
+        <f>PRODUCT(V4:V15)</f>
+        <v>212520</v>
+      </c>
+      <c r="W17">
+        <f>PRODUCT(W4:W15)</f>
+        <v>982080</v>
+      </c>
+      <c r="Y17">
+        <f>PRODUCT(Y4:Y15)</f>
+        <v>10626</v>
+      </c>
+      <c r="Z17">
+        <f>PRODUCT(Z4:Z15)</f>
+        <v>32736</v>
+      </c>
+      <c r="AB17">
+        <f>PRODUCT(AB4:AB15)</f>
+        <v>506</v>
+      </c>
+      <c r="AC17">
+        <f>PRODUCT(AC4:AC15)</f>
+        <v>1056</v>
+      </c>
+    </row>
+    <row r="18" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>0</v>
       </c>
-      <c r="B17" s="1">
-        <f>B16/C16</f>
+      <c r="B18" s="1">
+        <f>B17/C17</f>
         <v>3.810631341220885E-3</v>
       </c>
-      <c r="E17" s="1">
-        <f>E16/F16</f>
+      <c r="E18" s="1">
+        <f>E17/F17</f>
         <v>2.118878525997547E-2</v>
       </c>
-      <c r="H17" s="1">
-        <f>H16/I16</f>
+      <c r="H18" s="1">
+        <f>H17/I17</f>
         <v>9.1142936596218013E-2</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="K18" t="s">
+        <v>0</v>
+      </c>
+      <c r="L18" s="1">
+        <f>L17/M17</f>
+        <v>3.5314642099959118E-2</v>
+      </c>
+      <c r="O18" s="1">
+        <f>O17/P17</f>
+        <v>9.1142936596218013E-2</v>
+      </c>
+      <c r="R18" s="1">
+        <f>R17/S17</f>
+        <v>0.21639784946236559</v>
+      </c>
+      <c r="U18" t="s">
+        <v>0</v>
+      </c>
+      <c r="V18" s="1">
+        <f>V17/W17</f>
+        <v>0.21639784946236559</v>
+      </c>
+      <c r="Y18" s="1">
+        <f>Y17/Z17</f>
+        <v>0.32459677419354838</v>
+      </c>
+      <c r="AB18" s="1">
+        <f>AB17/AC17</f>
+        <v>0.47916666666666669</v>
+      </c>
+    </row>
+    <row r="19" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>8</v>
+      </c>
+      <c r="B19" s="4">
+        <f>1-B18</f>
+        <v>0.99618936865877916</v>
+      </c>
+      <c r="E19" s="4">
+        <f>1-E18</f>
+        <v>0.97881121474002453</v>
+      </c>
+      <c r="H19" s="4">
+        <f>1-H18</f>
+        <v>0.90885706340378203</v>
+      </c>
+      <c r="K19" t="s">
         <v>2</v>
       </c>
-      <c r="B18" s="1">
-        <f>1-B17</f>
-        <v>0.99618936865877916</v>
-      </c>
-      <c r="E18" s="1">
-        <f>1-E17</f>
-        <v>0.97881121474002453</v>
-      </c>
-      <c r="H18" s="1">
-        <f>1-H17</f>
+      <c r="L19" s="4">
+        <f>1-L18</f>
+        <v>0.96468535790004084</v>
+      </c>
+      <c r="O19" s="4">
+        <f>1-O18</f>
         <v>0.90885706340378203</v>
+      </c>
+      <c r="R19" s="4">
+        <f>1-R18</f>
+        <v>0.78360215053763438</v>
+      </c>
+      <c r="U19" t="s">
+        <v>2</v>
+      </c>
+      <c r="V19" s="4">
+        <f>1-V18</f>
+        <v>0.78360215053763438</v>
+      </c>
+      <c r="Y19" s="4">
+        <f>1-Y18</f>
+        <v>0.67540322580645162</v>
+      </c>
+      <c r="AB19" s="4">
+        <f>1-AB18</f>
+        <v>0.52083333333333326</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Faire un possible 3ème deck ; table des matières en page 2
</commit_message>
<xml_diff>
--- a/docs/Effet-de-Courroux-de-la-Terre.xlsx
+++ b/docs/Effet-de-Courroux-de-la-Terre.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leand\Documents\GitHub\Terre-de-Barons\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3426D6F-25AC-46D1-B13B-2D8E55DBD1B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B0D7013-B761-4394-886D-98FED9E22D59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-9120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="9">
   <si>
     <t>proba</t>
   </si>
@@ -60,9 +60,6 @@
   </si>
   <si>
     <t>2 positions tirées pour chaque événement calamité</t>
-  </si>
-  <si>
-    <t>prob cmp</t>
   </si>
   <si>
     <t>1 position tirée pour chaque événement calamité</t>
@@ -445,7 +442,7 @@
         <v>7</v>
       </c>
       <c r="U1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:29" x14ac:dyDescent="0.25">
@@ -1155,7 +1152,7 @@
     </row>
     <row r="19" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="B19" s="4">
         <f>1-B18</f>

</xml_diff>

<commit_message>
Calculs Gemini et raffinement du game design pour le second deck
</commit_message>
<xml_diff>
--- a/docs/Effet-de-Courroux-de-la-Terre.xlsx
+++ b/docs/Effet-de-Courroux-de-la-Terre.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leand\Documents\GitHub\Terre-de-Barons\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B0D7013-B761-4394-886D-98FED9E22D59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC04ED62-5F71-42AF-95C5-84A940FC32AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-9120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Courroux de la Terre" sheetId="1" r:id="rId1"/>
+    <sheet name="Gemini-1" sheetId="2" r:id="rId2"/>
+    <sheet name="Gemini-2" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="54">
   <si>
     <t>proba</t>
   </si>
@@ -63,16 +65,152 @@
   </si>
   <si>
     <t>1 position tirée pour chaque événement calamité</t>
+  </si>
+  <si>
+    <t>Nb de Donjons (K)</t>
+  </si>
+  <si>
+    <t>Moyenne théorique</t>
+  </si>
+  <si>
+    <t>Médiane (50% cumulé)</t>
+  </si>
+  <si>
+    <t>Quantile 90% (Pire cas)</t>
+  </si>
+  <si>
+    <t>2 joueurs (6 tirages)</t>
+  </si>
+  <si>
+    <t>8 Donjons</t>
+  </si>
+  <si>
+    <t>1,45</t>
+  </si>
+  <si>
+    <t>9 Donjons</t>
+  </si>
+  <si>
+    <t>1,64</t>
+  </si>
+  <si>
+    <t>10 Donjons</t>
+  </si>
+  <si>
+    <t>1,82</t>
+  </si>
+  <si>
+    <t>---</t>
+  </si>
+  <si>
+    <t>3 joueurs (9 tirages)</t>
+  </si>
+  <si>
+    <t>2,18</t>
+  </si>
+  <si>
+    <t>2,45</t>
+  </si>
+  <si>
+    <t>2,73</t>
+  </si>
+  <si>
+    <t>4 joueurs (12 tirages)</t>
+  </si>
+  <si>
+    <t>2,91</t>
+  </si>
+  <si>
+    <t>3,27</t>
+  </si>
+  <si>
+    <t>3,64</t>
+  </si>
+  <si>
+    <t>Q90/J</t>
+  </si>
+  <si>
+    <t>Nombre de joueurs (J)</t>
+  </si>
+  <si>
+    <t>Nombre de Joueurs (J)</t>
+  </si>
+  <si>
+    <t>Calamités / deck</t>
+  </si>
+  <si>
+    <t>Tirages max (n)</t>
+  </si>
+  <si>
+    <t>Tuiles occupées (T)</t>
+  </si>
+  <si>
+    <t>Moyenne globale</t>
+  </si>
+  <si>
+    <t>Moyenne / J</t>
+  </si>
+  <si>
+    <t>Médiane globale</t>
+  </si>
+  <si>
+    <t>Médiane / J</t>
+  </si>
+  <si>
+    <t>Quantile 90% global</t>
+  </si>
+  <si>
+    <t>Quantile 90% / J</t>
+  </si>
+  <si>
+    <t>J=2</t>
+  </si>
+  <si>
+    <t>5,09</t>
+  </si>
+  <si>
+    <t>2,55</t>
+  </si>
+  <si>
+    <t>2,5</t>
+  </si>
+  <si>
+    <t>3,5</t>
+  </si>
+  <si>
+    <t>J=3</t>
+  </si>
+  <si>
+    <t>8,73</t>
+  </si>
+  <si>
+    <t>3,67</t>
+  </si>
+  <si>
+    <t>J=4</t>
+  </si>
+  <si>
+    <t>6,55</t>
+  </si>
+  <si>
+    <t>1,75</t>
+  </si>
+  <si>
+    <t>2,25</t>
+  </si>
+  <si>
+    <t>Modèle : T = 10 + 2*J</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="0.0"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -94,6 +232,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -132,7 +276,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -140,6 +284,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1201,4 +1354,409 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEA1DF87-CCB7-4A16-BAD9-22262768D7EC}">
+  <dimension ref="B3:G14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="23.7109375" customWidth="1"/>
+    <col min="3" max="3" width="17.5703125" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="17.28515625" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:7" ht="26.25" x14ac:dyDescent="0.25">
+      <c r="B3" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="5">
+        <v>1</v>
+      </c>
+      <c r="F4" s="5">
+        <v>2</v>
+      </c>
+      <c r="G4" s="7">
+        <f>F4/2</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B5" s="5"/>
+      <c r="C5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="5">
+        <v>2</v>
+      </c>
+      <c r="F5" s="5">
+        <v>3</v>
+      </c>
+      <c r="G5" s="7">
+        <f t="shared" ref="G5:G6" si="0">F5/2</f>
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B6" s="5"/>
+      <c r="C6" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="5">
+        <v>2</v>
+      </c>
+      <c r="F6" s="5">
+        <v>3</v>
+      </c>
+      <c r="G6" s="7">
+        <f t="shared" si="0"/>
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B8" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="5">
+        <v>2</v>
+      </c>
+      <c r="F8" s="5">
+        <v>3</v>
+      </c>
+      <c r="G8" s="7">
+        <f>F8/3</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B9" s="5"/>
+      <c r="C9" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="5">
+        <v>2</v>
+      </c>
+      <c r="F9" s="5">
+        <v>4</v>
+      </c>
+      <c r="G9" s="7">
+        <f t="shared" ref="G9:G10" si="1">F9/3</f>
+        <v>1.3333333333333333</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B10" s="5"/>
+      <c r="C10" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="5">
+        <v>3</v>
+      </c>
+      <c r="F10" s="5">
+        <v>4</v>
+      </c>
+      <c r="G10" s="7">
+        <f t="shared" si="1"/>
+        <v>1.3333333333333333</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B11" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B12" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" s="5">
+        <v>3</v>
+      </c>
+      <c r="F12" s="5">
+        <v>4</v>
+      </c>
+      <c r="G12" s="7">
+        <f>F12/4</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B13" s="5"/>
+      <c r="C13" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" s="5">
+        <v>3</v>
+      </c>
+      <c r="F13" s="5">
+        <v>5</v>
+      </c>
+      <c r="G13" s="7">
+        <f t="shared" ref="G13:G14" si="2">F13/4</f>
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B14" s="5"/>
+      <c r="C14" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" s="5">
+        <v>4</v>
+      </c>
+      <c r="F14" s="5">
+        <v>5</v>
+      </c>
+      <c r="G14" s="7">
+        <f t="shared" si="2"/>
+        <v>1.25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AA82BD5-2B06-4C44-BE0D-627969746889}">
+  <dimension ref="B2:K9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="24.85546875" customWidth="1"/>
+    <col min="3" max="3" width="17.42578125" customWidth="1"/>
+    <col min="4" max="4" width="16.28515625" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="18.7109375" customWidth="1"/>
+    <col min="7" max="7" width="20.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:11" ht="39" x14ac:dyDescent="0.25">
+      <c r="B2" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B3" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="5">
+        <v>2</v>
+      </c>
+      <c r="D3" s="5">
+        <v>12</v>
+      </c>
+      <c r="E3" s="5">
+        <v>14</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="H3" s="5">
+        <v>5</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="J3" s="5">
+        <v>7</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B4" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="5">
+        <v>2</v>
+      </c>
+      <c r="D4" s="5">
+        <v>18</v>
+      </c>
+      <c r="E4" s="5">
+        <v>16</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" s="5">
+        <v>9</v>
+      </c>
+      <c r="I4" s="5">
+        <v>3</v>
+      </c>
+      <c r="J4" s="5">
+        <v>11</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B5" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="5">
+        <v>1</v>
+      </c>
+      <c r="D5" s="5">
+        <v>12</v>
+      </c>
+      <c r="E5" s="5">
+        <v>18</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" s="5">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="J5" s="5">
+        <v>9</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>53</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>